<commit_message>
Capping overtime to 2 hr/day instead of checking for monthly qouta
</commit_message>
<xml_diff>
--- a/tests/sample_export_UNPLANNED_result.xlsx
+++ b/tests/sample_export_UNPLANNED_result.xlsx
@@ -988,7 +988,7 @@
       </c>
       <c r="L6" s="6" t="inlineStr">
         <is>
-          <t>DEEPAK DEWAN</t>
+          <t>KARIM KHAN</t>
         </is>
       </c>
       <c r="M6" s="7" t="inlineStr">
@@ -1057,7 +1057,7 @@
       </c>
       <c r="L7" s="6" t="inlineStr">
         <is>
-          <t>KARIM KHAN</t>
+          <t>SHIB BAHADUR</t>
         </is>
       </c>
       <c r="M7" s="8" t="inlineStr">
@@ -1126,7 +1126,7 @@
       </c>
       <c r="L8" s="6" t="inlineStr">
         <is>
-          <t>KARIM KHAN</t>
+          <t>SHIB BAHADUR</t>
         </is>
       </c>
       <c r="M8" s="8" t="inlineStr">
@@ -1257,7 +1257,7 @@
       </c>
       <c r="L10" s="6" t="inlineStr">
         <is>
-          <t>SHIB BAHADUR</t>
+          <t>RAMIL ANCHETA MANALO</t>
         </is>
       </c>
       <c r="M10" s="6" t="n"/>
@@ -1321,7 +1321,7 @@
       </c>
       <c r="L11" s="6" t="inlineStr">
         <is>
-          <t>KARIM KHAN</t>
+          <t>SHIB BAHADUR</t>
         </is>
       </c>
       <c r="M11" s="8" t="inlineStr">
@@ -1452,7 +1452,7 @@
       </c>
       <c r="L13" s="6" t="inlineStr">
         <is>
-          <t>RAMIL ANCHETA MANALO</t>
+          <t>ARAVIND BALAKRISHNAN</t>
         </is>
       </c>
       <c r="M13" s="4" t="inlineStr">
@@ -1521,7 +1521,7 @@
       </c>
       <c r="L14" s="6" t="inlineStr">
         <is>
-          <t>RAMIL ANCHETA MANALO</t>
+          <t>ARAVIND BALAKRISHNAN</t>
         </is>
       </c>
       <c r="M14" s="4" t="inlineStr">
@@ -1719,14 +1719,10 @@
           <t>25 PAX MEP EQPTY BEV</t>
         </is>
       </c>
-      <c r="K17" s="6" t="inlineStr">
-        <is>
-          <t>T 82659</t>
-        </is>
-      </c>
+      <c r="K17" s="6" t="inlineStr"/>
       <c r="L17" s="6" t="inlineStr">
         <is>
-          <t>ARAVIND BALAKRISHNAN</t>
+          <t>AL SADAT HEAVY TRUCK</t>
         </is>
       </c>
       <c r="M17" s="11" t="inlineStr">
@@ -1788,14 +1784,10 @@
           <t>EQUIPMENT SHIFTING &amp; STAFF DROP</t>
         </is>
       </c>
-      <c r="K18" s="6" t="inlineStr">
-        <is>
-          <t>T 82659</t>
-        </is>
-      </c>
+      <c r="K18" s="6" t="inlineStr"/>
       <c r="L18" s="6" t="inlineStr">
         <is>
-          <t>ARAVIND BALAKRISHNAN</t>
+          <t>SAME AL SADAT HEAVY TRUCK</t>
         </is>
       </c>
       <c r="M18" s="11" t="inlineStr">
@@ -2066,7 +2058,7 @@
       </c>
       <c r="L22" s="6" t="inlineStr">
         <is>
-          <t>RAMIL ANCHETA MANALO</t>
+          <t>RASHEED THANDAPPURAM</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
@@ -2135,7 +2127,7 @@
       </c>
       <c r="L23" s="6" t="inlineStr">
         <is>
-          <t>AALIM HASSAN</t>
+          <t>KARIM KHAN</t>
         </is>
       </c>
       <c r="M23" s="12" t="inlineStr">
@@ -2400,7 +2392,7 @@
       </c>
       <c r="L27" s="6" t="inlineStr">
         <is>
-          <t>MANPREET SINGH</t>
+          <t>KARIM KHAN</t>
         </is>
       </c>
       <c r="M27" s="6" t="n"/>
@@ -2575,7 +2567,7 @@
       </c>
       <c r="L30" s="6" t="inlineStr">
         <is>
-          <t>IMRAN PASHA</t>
+          <t>MANPREET SINGH</t>
         </is>
       </c>
       <c r="M30" s="8" t="inlineStr">
@@ -2644,7 +2636,7 @@
       </c>
       <c r="L31" s="6" t="inlineStr">
         <is>
-          <t>IMRAN PASHA</t>
+          <t>MANPREET SINGH</t>
         </is>
       </c>
       <c r="M31" s="8" t="inlineStr">
@@ -2713,7 +2705,7 @@
       </c>
       <c r="L32" s="6" t="inlineStr">
         <is>
-          <t>IMRAN PASHA</t>
+          <t>MANPREET SINGH</t>
         </is>
       </c>
       <c r="M32" s="8" t="inlineStr">
@@ -2782,7 +2774,7 @@
       </c>
       <c r="L33" s="6" t="inlineStr">
         <is>
-          <t>IMRAN PASHA</t>
+          <t>MANPREET SINGH</t>
         </is>
       </c>
       <c r="M33" s="8" t="inlineStr">
@@ -2844,14 +2836,10 @@
           <t>CLEARANCE &amp; 2 STAFF PICKUP</t>
         </is>
       </c>
-      <c r="K34" s="6" t="inlineStr">
-        <is>
-          <t>B 50368</t>
-        </is>
-      </c>
+      <c r="K34" s="6" t="inlineStr"/>
       <c r="L34" s="6" t="inlineStr">
         <is>
-          <t>DEEPAK DEWAN</t>
+          <t>SAME AL SADAT HEAVY TRUCK</t>
         </is>
       </c>
       <c r="M34" s="7" t="inlineStr">
@@ -2920,7 +2908,7 @@
       </c>
       <c r="L35" s="6" t="inlineStr">
         <is>
-          <t>RASHEED THANDAPPURAM</t>
+          <t>DEEPAK DEWAN</t>
         </is>
       </c>
       <c r="M35" s="6" t="n"/>
@@ -2977,14 +2965,10 @@
           <t>EV ID # 602733 - 15th Feb - VVIP Ladies Dinner - Fatma Al Shamsi - FOOD PICK UP CHEF KAMAL WITH 2 CHEFS</t>
         </is>
       </c>
-      <c r="K36" s="6" t="inlineStr">
-        <is>
-          <t>B 50741</t>
-        </is>
-      </c>
+      <c r="K36" s="6" t="inlineStr"/>
       <c r="L36" s="6" t="inlineStr">
         <is>
-          <t>MUHAMMAD ATIF</t>
+          <t>AL WASL CHILLER TRUCK</t>
         </is>
       </c>
       <c r="M36" s="14" t="inlineStr">
@@ -3046,16 +3030,8 @@
           <t>15th ZLC - Ladies Wedding Ms. Aya Maher Abed Abu Shaireh - FOOD PICK UP @5PM - CHEF DISPATCH - CHEF ANTHONY</t>
         </is>
       </c>
-      <c r="K37" s="6" t="inlineStr">
-        <is>
-          <t>A 67338</t>
-        </is>
-      </c>
-      <c r="L37" s="6" t="inlineStr">
-        <is>
-          <t>AALIM HASSAN</t>
-        </is>
-      </c>
+      <c r="K37" s="6" t="inlineStr"/>
+      <c r="L37" s="6" t="inlineStr"/>
       <c r="M37" s="12" t="inlineStr">
         <is>
           <t>602649 - 602649 - 15th ZLC - Ladies
@@ -3122,7 +3098,7 @@
       </c>
       <c r="L38" s="6" t="inlineStr">
         <is>
-          <t>AALIM HASSAN</t>
+          <t>MUHAMMAD ATIF</t>
         </is>
       </c>
       <c r="M38" s="12" t="inlineStr">
@@ -3191,7 +3167,7 @@
       </c>
       <c r="L39" s="6" t="inlineStr">
         <is>
-          <t>IMRAN PASHA</t>
+          <t>RASHEED THANDAPPURAM</t>
         </is>
       </c>
       <c r="M39" s="8" t="inlineStr">
@@ -3253,14 +3229,10 @@
           <t>CLEARANCE &amp; STAFF PICKUP</t>
         </is>
       </c>
-      <c r="K40" s="6" t="inlineStr">
-        <is>
-          <t>T 82659</t>
-        </is>
-      </c>
+      <c r="K40" s="6" t="inlineStr"/>
       <c r="L40" s="6" t="inlineStr">
         <is>
-          <t>ARAVIND BALAKRISHNAN</t>
+          <t>SAME AL SADAT HEAVY TRUCK</t>
         </is>
       </c>
       <c r="M40" s="11" t="inlineStr">
@@ -3329,7 +3301,7 @@
       </c>
       <c r="L41" s="6" t="inlineStr">
         <is>
-          <t>MUHAMMAD ATIF</t>
+          <t>VISWANADHAN</t>
         </is>
       </c>
       <c r="M41" s="14" t="inlineStr">
@@ -3391,16 +3363,8 @@
           <t>15th ZLC - Ladies Wedding Ms. Aya Maher Abed Abu Shaireh - STAFF BUS @10PM - 5 CHEFS (RETURN BUS)</t>
         </is>
       </c>
-      <c r="K42" s="6" t="inlineStr">
-        <is>
-          <t>B 51850</t>
-        </is>
-      </c>
-      <c r="L42" s="6" t="inlineStr">
-        <is>
-          <t>AALIM HASSAN</t>
-        </is>
-      </c>
+      <c r="K42" s="6" t="inlineStr"/>
+      <c r="L42" s="6" t="inlineStr"/>
       <c r="M42" s="12" t="inlineStr">
         <is>
           <t>602649 - 602649 - 15th ZLC - Ladies
@@ -3460,16 +3424,8 @@
           <t>CLEARANCE &amp; 2 STAFF PICKUP + FOOD TRUCKS</t>
         </is>
       </c>
-      <c r="K43" s="6" t="inlineStr">
-        <is>
-          <t>A 67338</t>
-        </is>
-      </c>
-      <c r="L43" s="6" t="inlineStr">
-        <is>
-          <t>AALIM HASSAN</t>
-        </is>
-      </c>
+      <c r="K43" s="6" t="inlineStr"/>
+      <c r="L43" s="6" t="inlineStr"/>
       <c r="M43" s="12" t="inlineStr">
         <is>
           <t>602649 - 602649 - 15th ZLC - Ladies
@@ -3529,16 +3485,8 @@
           <t>CLEARANCE</t>
         </is>
       </c>
-      <c r="K44" s="6" t="inlineStr">
-        <is>
-          <t>A 67338</t>
-        </is>
-      </c>
-      <c r="L44" s="6" t="inlineStr">
-        <is>
-          <t>AALIM HASSAN</t>
-        </is>
-      </c>
+      <c r="K44" s="6" t="inlineStr"/>
+      <c r="L44" s="6" t="inlineStr"/>
       <c r="M44" s="12" t="inlineStr">
         <is>
           <t>602649 - 602649 - 15th ZLC - Ladies
@@ -3598,16 +3546,8 @@
           <t>18 STAFF TRANSPORTATION</t>
         </is>
       </c>
-      <c r="K45" s="6" t="inlineStr">
-        <is>
-          <t>B 51850</t>
-        </is>
-      </c>
-      <c r="L45" s="6" t="inlineStr">
-        <is>
-          <t>AALIM HASSAN</t>
-        </is>
-      </c>
+      <c r="K45" s="6" t="inlineStr"/>
+      <c r="L45" s="6" t="inlineStr"/>
       <c r="M45" s="12" t="inlineStr">
         <is>
           <t>602649 - 602649 - 15th ZLC - Ladies

</xml_diff>